<commit_message>
Release v1.0: Configuration Library Direct Mode
</commit_message>
<xml_diff>
--- a/Configuration Library/ACC_1.5MW_GASENGINE_CDU/equipment/CDU_2/CDU_2.xlsx
+++ b/Configuration Library/ACC_1.5MW_GASENGINE_CDU/equipment/CDU_2/CDU_2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ariel\Desktop\Configuration Library\ACC_1.5MW_GASENGINE_CDU\equipment\CDU_2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ArielLuoProjectspue-solver\Configuration Library\ACC_1.5MW_GASENGINE_CDU\equipment\CDU_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DB79947A-E33D-4A1C-9B61-21DB9E7EF293}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEEB68EB-FC49-485C-94CB-29D978B0E4F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -553,7 +553,7 @@
         <v>11</v>
       </c>
       <c r="B5">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C5" t="s">
         <v>12</v>
@@ -674,7 +674,7 @@
         <v>31</v>
       </c>
       <c r="B2">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s">
         <v>13</v>
@@ -703,7 +703,7 @@
         <v>0.1</v>
       </c>
       <c r="B2">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -711,7 +711,7 @@
         <v>0.2</v>
       </c>
       <c r="B3">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -719,7 +719,7 @@
         <v>0.3</v>
       </c>
       <c r="B4">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -727,7 +727,7 @@
         <v>0.4</v>
       </c>
       <c r="B5">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
@@ -735,7 +735,7 @@
         <v>0.5</v>
       </c>
       <c r="B6">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -743,7 +743,7 @@
         <v>0.6</v>
       </c>
       <c r="B7">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -751,7 +751,7 @@
         <v>0.7</v>
       </c>
       <c r="B8">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
@@ -759,7 +759,7 @@
         <v>0.8</v>
       </c>
       <c r="B9">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
@@ -767,7 +767,7 @@
         <v>0.9</v>
       </c>
       <c r="B10">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
@@ -775,7 +775,7 @@
         <v>1</v>
       </c>
       <c r="B11">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>